<commit_message>
docs: add cobol constitution and review gaps
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -6,7 +6,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Flows" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'User Flows'!$A$6:$N$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'User Flows'!$A$6:$N$38</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -696,7 +696,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -729,6 +729,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
         <is>
@@ -1435,7 +1436,7 @@
       </c>
       <c r="D16" s="77" t="inlineStr">
         <is>
-          <t>Deposit/withdrawal behavior is understood, but no COBOL migration SDD or target implementation exists yet.</t>
+          <t>Deposit/withdrawal behavior, validation quirks, missing-file failure, and unchecked shell persistence are understood, but no COBOL migration SDD or target implementation exists yet.</t>
         </is>
       </c>
       <c r="E16" s="77" t="n"/>
@@ -1745,7 +1746,7 @@
       </c>
       <c r="F21" s="80" t="inlineStr">
         <is>
-          <t>Console displays `Invalid Type.`; the account record is saved unchanged.</t>
+          <t>Console displays `Invalid Type.` and then misleadingly displays `Saving...`; the account balance remains unchanged but the file is still rewritten.</t>
         </is>
       </c>
       <c r="G21" s="80" t="inlineStr">
@@ -1755,7 +1756,7 @@
       </c>
       <c r="H21" s="80" t="inlineStr">
         <is>
-          <t>TRANS-PROC.CBL ELSE branch after D/W checks DISPLAY 'Invalid Type.'; unchanged ACCOUNT-REC is written to TEMP-REC.</t>
+          <t>TRANS-PROC.CBL sets WS-FOUND-FLAG = 'Y' before validating type; invalid type branch DISPLAY 'Invalid Type.' leaves ACCOUNT-REC unchanged; final IF WS-FOUND-FLAG = 'Y' displays 'Saving...' and swaps ACCOUNTS.TMP into ACCOUNTS.DAT.</t>
         </is>
       </c>
       <c r="I21" s="80" t="inlineStr">
@@ -1765,7 +1766,7 @@
       </c>
       <c r="J21" s="80" t="inlineStr">
         <is>
-          <t>No migrated invalid-type validation exists yet.</t>
+          <t>No migrated invalid-type behavior exists yet; SDD must decide whether to preserve the misleading `Saving...` message or intentionally improve it.</t>
         </is>
       </c>
       <c r="K21" s="80" t="inlineStr">
@@ -1925,63 +1926,99 @@
         </is>
       </c>
     </row>
-    <row r="24" collapsed="1" ht="66" customHeight="1">
-      <c r="A24" s="77" t="inlineStr">
-        <is>
-          <t>UF-004</t>
-        </is>
-      </c>
-      <c r="B24" s="77" t="inlineStr">
-        <is>
-          <t>Account Balance Reporting</t>
-        </is>
-      </c>
-      <c r="C24" s="77" t="inlineStr">
-        <is>
-          <t>Not Passed - Missed</t>
-        </is>
-      </c>
-      <c r="D24" s="77" t="inlineStr">
-        <is>
-          <t>Legacy reporting behavior is understood, but no COBOL migration SDD or target implementation exists yet.</t>
-        </is>
-      </c>
-      <c r="E24" s="77" t="n"/>
-      <c r="F24" s="77" t="n"/>
-      <c r="G24" s="77" t="n"/>
-      <c r="H24" s="77" t="n"/>
-      <c r="I24" s="77" t="n"/>
-      <c r="J24" s="77" t="n"/>
-      <c r="K24" s="77" t="n"/>
-      <c r="L24" s="77" t="n"/>
-      <c r="M24" s="77" t="n"/>
-      <c r="N24" s="77" t="n"/>
-    </row>
-    <row r="25" hidden="1" outlineLevel="1" collapsed="1" ht="37.5" customHeight="1">
+    <row r="24" hidden="1" outlineLevel="1" ht="66" customHeight="1">
+      <c r="A24" s="78" t="n"/>
+      <c r="B24" s="79" t="inlineStr">
+        <is>
+          <t>Missing transaction file</t>
+        </is>
+      </c>
+      <c r="C24" s="78" t="inlineStr">
+        <is>
+          <t>Alternative path</t>
+        </is>
+      </c>
+      <c r="D24" s="80" t="inlineStr">
+        <is>
+          <t>Starting a transaction without ACCOUNTS.DAT shall fall through to COBOL runtime/file handling because TRANS-PROC has no custom missing-file recovery.</t>
+        </is>
+      </c>
+      <c r="E24" s="80" t="inlineStr">
+        <is>
+          <t>The legacy operator must run Init Database before transactions; otherwise the terminal program does not provide a business-friendly recovery path.</t>
+        </is>
+      </c>
+      <c r="F24" s="80" t="inlineStr">
+        <is>
+          <t>The program fails at/opening the input account file rather than showing a domain validation message.</t>
+        </is>
+      </c>
+      <c r="G24" s="80" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H24" s="80" t="inlineStr">
+        <is>
+          <t>TRANS-PROC.CBL OPEN INPUT ACCOUNT-FILE has no INVALID KEY/USE AFTER ERROR/custom exception branch; ACCOUNT-FILE is assigned to 'ACCOUNTS.DAT'.</t>
+        </is>
+      </c>
+      <c r="I24" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J24" s="80" t="inlineStr">
+        <is>
+          <t>No migrated missing-file behavior exists yet; SDD should decide whether to preserve runtime failure or improve it with an explicit error.</t>
+        </is>
+      </c>
+      <c r="K24" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L24" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M24" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N24" s="80" t="inlineStr">
+        <is>
+          <t>No COBOL .specify/memory/constitution.md or specs/ SDD artifacts existed when this row was captured; constitution was added on 2026-07-09 and feature specs are still pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" hidden="1" outlineLevel="1" ht="37.5" customHeight="1">
       <c r="A25" s="78" t="n"/>
       <c r="B25" s="79" t="inlineStr">
         <is>
-          <t>Print account balance report</t>
+          <t>Unchecked shell persistence</t>
         </is>
       </c>
       <c r="C25" s="78" t="inlineStr">
         <is>
-          <t>Happy path</t>
+          <t>Operational path</t>
         </is>
       </c>
       <c r="D25" s="80" t="inlineStr">
         <is>
-          <t>The report command shall print every account's number, customer name, and formatted balance.</t>
+          <t>Transaction persistence depends on shell commands and does not check their return status.</t>
         </is>
       </c>
       <c r="E25" s="80" t="inlineStr">
         <is>
-          <t>A user can inspect the current balances in the flat-file database.</t>
+          <t>The legacy save path can claim success even if deleting or moving the account file fails due to platform or permission problems.</t>
         </is>
       </c>
       <c r="F25" s="80" t="inlineStr">
         <is>
-          <t>Console displays `--- ACCOUNT BALANCE SUMMARY REPORT ---`, a header, then each account number, name, and currency-formatted balance.</t>
+          <t>Console displays `Saving...`; if `rm`/`mv` fails, the program has no user-visible failure handling in COBOL.</t>
         </is>
       </c>
       <c r="G25" s="80" t="inlineStr">
@@ -1991,7 +2028,7 @@
       </c>
       <c r="H25" s="80" t="inlineStr">
         <is>
-          <t>REPORT-GEN.CBL DISPLAY report title/header; READ ACCOUNT-FILE until EOF; DISPLAY REC-ACC-NUMBER, REC-ACC-NAME, WS-FORMATTED-BAL.</t>
+          <t>TRANS-PROC.CBL CALL 'SYSTEM' USING WS-CMD for 'rm -f ACCOUNTS.DAT' and 'mv ACCOUNTS.TMP ACCOUNTS.DAT'; no return-code/status check follows either call. Original upstream used Windows `cmd /c del`/`ren`; Docker baseline uses Linux commands.</t>
         </is>
       </c>
       <c r="I25" s="80" t="inlineStr">
@@ -2001,7 +2038,7 @@
       </c>
       <c r="J25" s="80" t="inlineStr">
         <is>
-          <t>No migrated report view/API exists yet.</t>
+          <t>No migrated persistence strategy exists yet; target should use checked persistence APIs/transactions and document this as an intentional legacy improvement.</t>
         </is>
       </c>
       <c r="K25" s="80" t="inlineStr">
@@ -2021,103 +2058,67 @@
       </c>
       <c r="N25" s="80" t="inlineStr">
         <is>
-          <t>No COBOL .specify/memory/constitution.md or specs/ SDD artifacts exist yet in this repo as of 2026-07-09.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" hidden="1" outlineLevel="1" ht="66" customHeight="1">
-      <c r="A26" s="78" t="n"/>
-      <c r="B26" s="79" t="inlineStr">
-        <is>
-          <t>Calculate report totals</t>
-        </is>
-      </c>
-      <c r="C26" s="78" t="inlineStr">
-        <is>
-          <t>Happy path</t>
-        </is>
-      </c>
-      <c r="D26" s="80" t="inlineStr">
-        <is>
-          <t>The report shall show the total number of accounts and total bank balance across all records.</t>
-        </is>
-      </c>
-      <c r="E26" s="80" t="inlineStr">
-        <is>
-          <t>The report gives an operator a quick aggregate view of the account file.</t>
-        </is>
-      </c>
-      <c r="F26" s="80" t="inlineStr">
-        <is>
-          <t>Console displays `TOTAL ACCOUNTS: 00003` and `BANK BALANCE: $ ...` for the current file contents.</t>
-        </is>
-      </c>
-      <c r="G26" s="80" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H26" s="80" t="inlineStr">
-        <is>
-          <t>REPORT-GEN.CBL ADD REC-ACC-BALANCE TO WS-TOTAL-BAL; ADD 1 TO WS-COUNT; DISPLAY totals after CLOSE ACCOUNT-FILE.</t>
-        </is>
-      </c>
-      <c r="I26" s="80" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J26" s="80" t="inlineStr">
-        <is>
-          <t>No migrated aggregate report exists yet.</t>
-        </is>
-      </c>
-      <c r="K26" s="80" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L26" s="80" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M26" s="80" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N26" s="80" t="inlineStr">
-        <is>
-          <t>No COBOL .specify/memory/constitution.md or specs/ SDD artifacts exist yet in this repo as of 2026-07-09.</t>
-        </is>
-      </c>
+          <t>No COBOL .specify/memory/constitution.md or specs/ SDD artifacts existed when this row was captured; constitution was added on 2026-07-09 and feature specs are still pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" collapsed="1" ht="66" customHeight="1">
+      <c r="A26" s="77" t="inlineStr">
+        <is>
+          <t>UF-004</t>
+        </is>
+      </c>
+      <c r="B26" s="77" t="inlineStr">
+        <is>
+          <t>Account Balance Reporting</t>
+        </is>
+      </c>
+      <c r="C26" s="77" t="inlineStr">
+        <is>
+          <t>Not Passed - Missed</t>
+        </is>
+      </c>
+      <c r="D26" s="77" t="inlineStr">
+        <is>
+          <t>Legacy reporting behavior, including its vertical terminal layout, is understood, but no COBOL migration SDD or target implementation exists yet.</t>
+        </is>
+      </c>
+      <c r="E26" s="77" t="n"/>
+      <c r="F26" s="77" t="n"/>
+      <c r="G26" s="77" t="n"/>
+      <c r="H26" s="77" t="n"/>
+      <c r="I26" s="77" t="n"/>
+      <c r="J26" s="77" t="n"/>
+      <c r="K26" s="77" t="n"/>
+      <c r="L26" s="77" t="n"/>
+      <c r="M26" s="77" t="n"/>
+      <c r="N26" s="77" t="n"/>
     </row>
     <row r="27" hidden="1" outlineLevel="1" ht="66" customHeight="1">
       <c r="A27" s="78" t="n"/>
       <c r="B27" s="79" t="inlineStr">
         <is>
-          <t>Repeat report after transactions</t>
+          <t>Print account balance report</t>
         </is>
       </c>
       <c r="C27" s="78" t="inlineStr">
         <is>
-          <t>Operational path</t>
+          <t>Happy path</t>
         </is>
       </c>
       <c r="D27" s="80" t="inlineStr">
         <is>
-          <t>Repeated report calls in the same menu session shall recalculate totals from the account file rather than reuse stale working-storage values.</t>
+          <t>The report command shall print every account's number, customer name, and formatted balance as the legacy terminal actually renders them: vertical account blocks, despite a tabular-looking header.</t>
         </is>
       </c>
       <c r="E27" s="80" t="inlineStr">
         <is>
-          <t>After deposits or withdrawals, the operator can rerun the report and see fresh totals.</t>
+          <t>The report gives a user a current balance view, but the visual layout is not a real table: the header says `NUM | NAME | BALANCE`, while each account prints across separate lines.</t>
         </is>
       </c>
       <c r="F27" s="80" t="inlineStr">
         <is>
-          <t>A second report after a transaction reflects the changed balance and bank total.</t>
+          <t>Console displays the report title/header, then for each account prints account number, name, formatted balance, and a blank line.</t>
         </is>
       </c>
       <c r="G27" s="80" t="inlineStr">
@@ -2127,7 +2128,7 @@
       </c>
       <c r="H27" s="80" t="inlineStr">
         <is>
-          <t>REPORT-GEN.CBL MAIN-PROCEDURE resets WS-EOF-FLAG, WS-TOTAL-BAL, and WS-COUNT before OPEN INPUT ACCOUNT-FILE; validated by docker demo flow in README.demo.md.</t>
+          <t>REPORT-GEN.CBL DISPLAY 'NUM | NAME | BALANCE'; inside the READ loop it separately DISPLAYs REC-ACC-NUMBER, REC-ACC-NAME, WS-FORMATTED-BAL, and DISPLAY ' '.</t>
         </is>
       </c>
       <c r="I27" s="80" t="inlineStr">
@@ -2137,7 +2138,7 @@
       </c>
       <c r="J27" s="80" t="inlineStr">
         <is>
-          <t>No migrated state-reset/report-refresh behavior exists yet.</t>
+          <t>No migrated report view/API exists yet; SDD must decide whether a target UI preserves the vertical legacy output or documents a table-layout modernization.</t>
         </is>
       </c>
       <c r="K27" s="80" t="inlineStr">
@@ -2165,37 +2166,37 @@
       <c r="A28" s="78" t="n"/>
       <c r="B28" s="79" t="inlineStr">
         <is>
-          <t>Missing account file behavior</t>
+          <t>Calculate report totals</t>
         </is>
       </c>
       <c r="C28" s="78" t="inlineStr">
         <is>
-          <t>Alternative path</t>
+          <t>Happy path</t>
         </is>
       </c>
       <c r="D28" s="80" t="inlineStr">
         <is>
-          <t>The legacy report has no custom business error message when ACCOUNTS.DAT is absent.</t>
+          <t>The report shall show the total number of accounts and total bank balance across all records.</t>
         </is>
       </c>
       <c r="E28" s="80" t="inlineStr">
         <is>
-          <t>Operators must initialize the file before using report; missing-file recovery is not part of the legacy UI flow.</t>
+          <t>The report gives an operator a quick aggregate view of the account file.</t>
         </is>
       </c>
       <c r="F28" s="80" t="inlineStr">
         <is>
-          <t>If the file is absent, behavior falls through to COBOL runtime/file handling rather than a user-friendly business message.</t>
+          <t>Console displays `TOTAL ACCOUNTS: 00003` and `BANK BALANCE: $ ...` for the current file contents.</t>
         </is>
       </c>
       <c r="G28" s="80" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H28" s="80" t="inlineStr">
         <is>
-          <t>REPORT-GEN.CBL OPEN INPUT ACCOUNT-FILE has no INVALID KEY/USE AFTER ERROR/custom exception branch; INIT-DB is the expected prior setup path.</t>
+          <t>REPORT-GEN.CBL ADD REC-ACC-BALANCE TO WS-TOTAL-BAL; ADD 1 TO WS-COUNT; DISPLAY totals after CLOSE ACCOUNT-FILE.</t>
         </is>
       </c>
       <c r="I28" s="80" t="inlineStr">
@@ -2205,7 +2206,7 @@
       </c>
       <c r="J28" s="80" t="inlineStr">
         <is>
-          <t>No migrated missing-file handling decision exists yet.</t>
+          <t>No migrated aggregate report exists yet.</t>
         </is>
       </c>
       <c r="K28" s="80" t="inlineStr">
@@ -2229,73 +2230,109 @@
         </is>
       </c>
     </row>
-    <row r="29" collapsed="1" ht="66" customHeight="1">
-      <c r="A29" s="77" t="inlineStr">
-        <is>
-          <t>UF-005</t>
-        </is>
-      </c>
-      <c r="B29" s="77" t="inlineStr">
-        <is>
-          <t>Account Record Model &amp; Status Codes</t>
-        </is>
-      </c>
-      <c r="C29" s="77" t="inlineStr">
-        <is>
-          <t>Not Passed - Missed</t>
-        </is>
-      </c>
-      <c r="D29" s="77" t="inlineStr">
-        <is>
-          <t>Legacy data shape is understood, but no COBOL migration SDD or target implementation exists yet.</t>
-        </is>
-      </c>
-      <c r="E29" s="77" t="n"/>
-      <c r="F29" s="77" t="n"/>
-      <c r="G29" s="77" t="n"/>
-      <c r="H29" s="77" t="n"/>
-      <c r="I29" s="77" t="n"/>
-      <c r="J29" s="77" t="n"/>
-      <c r="K29" s="77" t="n"/>
-      <c r="L29" s="77" t="n"/>
-      <c r="M29" s="77" t="n"/>
-      <c r="N29" s="77" t="n"/>
+    <row r="29" hidden="1" outlineLevel="1" ht="66" customHeight="1">
+      <c r="A29" s="78" t="n"/>
+      <c r="B29" s="79" t="inlineStr">
+        <is>
+          <t>Repeat report after transactions</t>
+        </is>
+      </c>
+      <c r="C29" s="78" t="inlineStr">
+        <is>
+          <t>Operational path</t>
+        </is>
+      </c>
+      <c r="D29" s="80" t="inlineStr">
+        <is>
+          <t>Repeated report calls in the same menu session shall recalculate totals from the account file rather than reuse stale working-storage values.</t>
+        </is>
+      </c>
+      <c r="E29" s="80" t="inlineStr">
+        <is>
+          <t>After deposits or withdrawals, the operator can rerun the report and see fresh totals.</t>
+        </is>
+      </c>
+      <c r="F29" s="80" t="inlineStr">
+        <is>
+          <t>A second report after a transaction reflects the changed balance and bank total.</t>
+        </is>
+      </c>
+      <c r="G29" s="80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H29" s="80" t="inlineStr">
+        <is>
+          <t>REPORT-GEN.CBL MAIN-PROCEDURE resets WS-EOF-FLAG, WS-TOTAL-BAL, and WS-COUNT before OPEN INPUT ACCOUNT-FILE; validated by docker demo flow in README.demo.md.</t>
+        </is>
+      </c>
+      <c r="I29" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J29" s="80" t="inlineStr">
+        <is>
+          <t>No migrated state-reset/report-refresh behavior exists yet.</t>
+        </is>
+      </c>
+      <c r="K29" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L29" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M29" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N29" s="80" t="inlineStr">
+        <is>
+          <t>No COBOL .specify/memory/constitution.md or specs/ SDD artifacts exist yet in this repo as of 2026-07-09.</t>
+        </is>
+      </c>
     </row>
     <row r="30" hidden="1" outlineLevel="1" ht="66" customHeight="1">
       <c r="A30" s="78" t="n"/>
       <c r="B30" s="79" t="inlineStr">
         <is>
-          <t>Account record fields</t>
+          <t>Missing account file behavior</t>
         </is>
       </c>
       <c r="C30" s="78" t="inlineStr">
         <is>
-          <t>Operational path</t>
+          <t>Alternative path</t>
         </is>
       </c>
       <c r="D30" s="80" t="inlineStr">
         <is>
-          <t>Account records shall carry account number, customer name, signed decimal balance, and one-character status.</t>
+          <t>The legacy report has no custom business error message when ACCOUNTS.DAT is absent.</t>
         </is>
       </c>
       <c r="E30" s="80" t="inlineStr">
         <is>
-          <t>These fields are the minimum data contract shared by initialization, transaction processing, and reporting.</t>
+          <t>Operators must initialize the file before using report; missing-file recovery is not part of the legacy UI flow.</t>
         </is>
       </c>
       <c r="F30" s="80" t="inlineStr">
         <is>
-          <t>The flat file stores numeric account ids, fixed-width names, balances, and status values used by the COBOL programs.</t>
+          <t>If the file is absent, behavior falls through to COBOL runtime/file handling rather than a user-friendly business message.</t>
         </is>
       </c>
       <c r="G30" s="80" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="H30" s="80" t="inlineStr">
         <is>
-          <t>ACCOUNTS.CPY ACCOUNT-RECORD fields ACC-NUMBER, ACC-CUSTOMER-NAME, ACC-BALANCE, ACC-STATUS; INIT-DB.CBL/TRANS-PROC.CBL/REPORT-GEN.CBL FD ACCOUNT-REC mirrors these fields.</t>
+          <t>REPORT-GEN.CBL OPEN INPUT ACCOUNT-FILE has no INVALID KEY/USE AFTER ERROR/custom exception branch; INIT-DB is the expected prior setup path.</t>
         </is>
       </c>
       <c r="I30" s="80" t="inlineStr">
@@ -2305,7 +2342,7 @@
       </c>
       <c r="J30" s="80" t="inlineStr">
         <is>
-          <t>No migrated domain model exists yet.</t>
+          <t>No migrated missing-file handling decision exists yet.</t>
         </is>
       </c>
       <c r="K30" s="80" t="inlineStr">
@@ -2329,109 +2366,73 @@
         </is>
       </c>
     </row>
-    <row r="31" hidden="1" outlineLevel="1" ht="66" customHeight="1">
-      <c r="A31" s="78" t="n"/>
-      <c r="B31" s="79" t="inlineStr">
-        <is>
-          <t>Active account seed status</t>
-        </is>
-      </c>
-      <c r="C31" s="78" t="inlineStr">
-        <is>
-          <t>Operational path</t>
-        </is>
-      </c>
-      <c r="D31" s="80" t="inlineStr">
-        <is>
-          <t>Initialized demo accounts shall be written with active status A.</t>
-        </is>
-      </c>
-      <c r="E31" s="80" t="inlineStr">
-        <is>
-          <t>The initial demo dataset treats every seeded customer account as active.</t>
-        </is>
-      </c>
-      <c r="F31" s="80" t="inlineStr">
-        <is>
-          <t>Each initialized account record has status `A`.</t>
-        </is>
-      </c>
-      <c r="G31" s="80" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H31" s="80" t="inlineStr">
-        <is>
-          <t>INIT-DB.CBL MOVE 'A' TO REC-ACC-STATUS before each WRITE ACCOUNT-REC.</t>
-        </is>
-      </c>
-      <c r="I31" s="80" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J31" s="80" t="inlineStr">
-        <is>
-          <t>No migrated seed/domain status behavior exists yet.</t>
-        </is>
-      </c>
-      <c r="K31" s="80" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L31" s="80" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M31" s="80" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N31" s="80" t="inlineStr">
-        <is>
-          <t>No COBOL .specify/memory/constitution.md or specs/ SDD artifacts exist yet in this repo as of 2026-07-09.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" hidden="1" outlineLevel="1" collapsed="1" ht="37.5" customHeight="1">
+    <row r="31" collapsed="1" ht="66" customHeight="1">
+      <c r="A31" s="77" t="inlineStr">
+        <is>
+          <t>UF-005</t>
+        </is>
+      </c>
+      <c r="B31" s="77" t="inlineStr">
+        <is>
+          <t>Account Record Model &amp; Status Codes</t>
+        </is>
+      </c>
+      <c r="C31" s="77" t="inlineStr">
+        <is>
+          <t>Not Passed - Missed</t>
+        </is>
+      </c>
+      <c r="D31" s="77" t="inlineStr">
+        <is>
+          <t>Legacy data-shape evidence is understood, including the unused/conflicting copybook, but no COBOL migration SDD or target implementation exists yet.</t>
+        </is>
+      </c>
+      <c r="E31" s="77" t="n"/>
+      <c r="F31" s="77" t="n"/>
+      <c r="G31" s="77" t="n"/>
+      <c r="H31" s="77" t="n"/>
+      <c r="I31" s="77" t="n"/>
+      <c r="J31" s="77" t="n"/>
+      <c r="K31" s="77" t="n"/>
+      <c r="L31" s="77" t="n"/>
+      <c r="M31" s="77" t="n"/>
+      <c r="N31" s="77" t="n"/>
+    </row>
+    <row r="32" hidden="1" outlineLevel="1" ht="37.5" customHeight="1">
       <c r="A32" s="78" t="n"/>
       <c r="B32" s="79" t="inlineStr">
         <is>
-          <t>Closed and suspended status vocabulary</t>
+          <t>Account record fields</t>
         </is>
       </c>
       <c r="C32" s="78" t="inlineStr">
         <is>
-          <t>Alternative path</t>
+          <t>Operational path</t>
         </is>
       </c>
       <c r="D32" s="80" t="inlineStr">
         <is>
-          <t>The copybook defines closed and suspended account status values, but runtime transaction/report behavior does not enforce them.</t>
+          <t>The active account record contract shall be taken from the inline FD layouts used by the executable programs, not from ACCOUNTS.CPY alone.</t>
         </is>
       </c>
       <c r="E32" s="80" t="inlineStr">
         <is>
-          <t>The data contract hints at future or unused account lifecycle states that a migration must decide to preserve, implement, or defer.</t>
+          <t>The running programs duplicate ACCOUNT-REC inline. ACCOUNTS.CPY exists but is not included by any active program and therefore cannot be treated as the persistence source of truth without reconciliation.</t>
         </is>
       </c>
       <c r="F32" s="80" t="inlineStr">
         <is>
-          <t>No user-visible branch changes for C/S statuses are implemented in the current programs.</t>
+          <t>The flat file stores numeric account ids, fixed-width names, display numeric balances, and status values as read/written by INIT-DB, TRANS-PROC, and REPORT-GEN.</t>
         </is>
       </c>
       <c r="G32" s="80" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H32" s="80" t="inlineStr">
         <is>
-          <t>ACCOUNTS.CPY defines 88-level ACC-ACTIVE='A', ACC-CLOSED='C', ACC-SUSPENDED='S'; TRANS-PROC.CBL and REPORT-GEN.CBL do not check REC-ACC-STATUS.</t>
+          <t>INIT-DB.CBL, TRANS-PROC.CBL, and REPORT-GEN.CBL each declare FD ACCOUNT-FILE / 01 ACCOUNT-REC inline; no active program contains COPY ACCOUNTS.CPY.</t>
         </is>
       </c>
       <c r="I32" s="80" t="inlineStr">
@@ -2441,7 +2442,7 @@
       </c>
       <c r="J32" s="80" t="inlineStr">
         <is>
-          <t>No migrated status decision exists yet.</t>
+          <t>No migrated domain model exists yet; SDD must explicitly choose the active inline FD/display numeric contract or document a conversion.</t>
         </is>
       </c>
       <c r="K32" s="80" t="inlineStr">
@@ -2465,73 +2466,109 @@
         </is>
       </c>
     </row>
-    <row r="33" collapsed="1" ht="66" customHeight="1">
-      <c r="A33" s="77" t="inlineStr">
-        <is>
-          <t>UF-006</t>
-        </is>
-      </c>
-      <c r="B33" s="77" t="inlineStr">
-        <is>
-          <t>Legacy Runtime &amp; Demo Deployment</t>
-        </is>
-      </c>
-      <c r="C33" s="77" t="inlineStr">
-        <is>
-          <t>Not Passed - Missed</t>
-        </is>
-      </c>
-      <c r="D33" s="77" t="inlineStr">
-        <is>
-          <t>Dockerized legacy runtime exists for evidence gathering, but no migration SDD or target runtime decision exists yet.</t>
-        </is>
-      </c>
-      <c r="E33" s="77" t="n"/>
-      <c r="F33" s="77" t="n"/>
-      <c r="G33" s="77" t="n"/>
-      <c r="H33" s="77" t="n"/>
-      <c r="I33" s="77" t="n"/>
-      <c r="J33" s="77" t="n"/>
-      <c r="K33" s="77" t="n"/>
-      <c r="L33" s="77" t="n"/>
-      <c r="M33" s="77" t="n"/>
-      <c r="N33" s="77" t="n"/>
+    <row r="33" hidden="1" outlineLevel="1" ht="66" customHeight="1">
+      <c r="A33" s="78" t="n"/>
+      <c r="B33" s="79" t="inlineStr">
+        <is>
+          <t>Active account seed status</t>
+        </is>
+      </c>
+      <c r="C33" s="78" t="inlineStr">
+        <is>
+          <t>Operational path</t>
+        </is>
+      </c>
+      <c r="D33" s="80" t="inlineStr">
+        <is>
+          <t>Initialized demo accounts shall be written with active status A.</t>
+        </is>
+      </c>
+      <c r="E33" s="80" t="inlineStr">
+        <is>
+          <t>The initial demo dataset treats every seeded customer account as active.</t>
+        </is>
+      </c>
+      <c r="F33" s="80" t="inlineStr">
+        <is>
+          <t>Each initialized account record has status `A`.</t>
+        </is>
+      </c>
+      <c r="G33" s="80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H33" s="80" t="inlineStr">
+        <is>
+          <t>INIT-DB.CBL MOVE 'A' TO REC-ACC-STATUS before each WRITE ACCOUNT-REC.</t>
+        </is>
+      </c>
+      <c r="I33" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J33" s="80" t="inlineStr">
+        <is>
+          <t>No migrated seed/domain status behavior exists yet.</t>
+        </is>
+      </c>
+      <c r="K33" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L33" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M33" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N33" s="80" t="inlineStr">
+        <is>
+          <t>No COBOL .specify/memory/constitution.md or specs/ SDD artifacts exist yet in this repo as of 2026-07-09.</t>
+        </is>
+      </c>
     </row>
     <row r="34" hidden="1" outlineLevel="1" ht="66" customHeight="1">
       <c r="A34" s="78" t="n"/>
       <c r="B34" s="79" t="inlineStr">
         <is>
-          <t>Compile COBOL modules</t>
+          <t>Closed and suspended status vocabulary</t>
         </is>
       </c>
       <c r="C34" s="78" t="inlineStr">
         <is>
-          <t>Operational path</t>
+          <t>Alternative path</t>
         </is>
       </c>
       <c r="D34" s="80" t="inlineStr">
         <is>
-          <t>The demo runtime shall compile INIT-DB, TRANS-PROC, REPORT-GEN as modules and BANK-MAIN as the executable menu program.</t>
+          <t>ACCOUNTS.CPY defines status vocabulary and a COMP-3 balance field, but it is an unused/conflicting artifact in the current runtime.</t>
         </is>
       </c>
       <c r="E34" s="80" t="inlineStr">
         <is>
-          <t>A reviewer can rebuild the legacy baseline consistently without installing GnuCOBOL on Windows.</t>
+          <t>The copybook hints at account lifecycle states and packed decimal storage, but the executable programs neither include it nor enforce those statuses.</t>
         </is>
       </c>
       <c r="F34" s="80" t="inlineStr">
         <is>
-          <t>Docker build produces runnable COBOL artifacts inside the container.</t>
+          <t>No user-visible branch changes for C/S statuses are implemented; using ACCOUNTS.CPY's COMP-3 balance as-is would not match the line-sequential text file produced by INIT-DB.</t>
         </is>
       </c>
       <c r="G34" s="80" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="H34" s="80" t="inlineStr">
         <is>
-          <t>Dockerfile installs gnucobol/make and runs cobc -m INIT-DB.CBL, cobc -m TRANS-PROC.CBL, cobc -m REPORT-GEN.CBL, cobc -x BANK-MAIN.CBL.</t>
+          <t>ACCOUNTS.CPY defines ACC-BALANCE PIC S9(13)V99 COMP-3 and 88-level ACC-ACTIVE/ACC-CLOSED/ACC-SUSPENDED; active programs redeclare REC-ACC-BALANCE PIC S9(13)V99 and do not COPY the copybook.</t>
         </is>
       </c>
       <c r="I34" s="80" t="inlineStr">
@@ -2541,7 +2578,7 @@
       </c>
       <c r="J34" s="80" t="inlineStr">
         <is>
-          <t>No target deployment architecture exists for a migrated COBOL replacement yet.</t>
+          <t>No migrated status/storage decision exists yet; SDD must treat this as a migration decision, not a simple copybook import.</t>
         </is>
       </c>
       <c r="K34" s="80" t="inlineStr">
@@ -2569,73 +2606,238 @@
       <c r="A35" s="78" t="n"/>
       <c r="B35" s="79" t="inlineStr">
         <is>
+          <t>Copybook storage mismatch</t>
+        </is>
+      </c>
+      <c r="C35" s="78" t="inlineStr">
+        <is>
+          <t>Operational path</t>
+        </is>
+      </c>
+      <c r="D35" s="80" t="inlineStr">
+        <is>
+          <t>Migration analysis shall not import ACCOUNTS.CPY's COMP-3 balance definition as the active file format without conversion evidence.</t>
+        </is>
+      </c>
+      <c r="E35" s="80" t="inlineStr">
+        <is>
+          <t>The apparent copybook contract conflicts with the actual line-sequential file used by the running programs, so blindly following the copybook would corrupt or misread balances.</t>
+        </is>
+      </c>
+      <c r="F35" s="80" t="inlineStr">
+        <is>
+          <t>The active demo flow reads and writes display numeric balances in ACCOUNTS.DAT; ACCOUNTS.CPY is unused and conflicting.</t>
+        </is>
+      </c>
+      <c r="G35" s="80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H35" s="80" t="inlineStr">
+        <is>
+          <t>ACCOUNTS.CPY ACC-BALANCE PIC S9(13)V99 COMP-3; INIT-DB.CBL/TRANS-PROC.CBL/REPORT-GEN.CBL inline REC-ACC-BALANCE PIC S9(13)V99; no COPY ACCOUNTS.CPY statement found.</t>
+        </is>
+      </c>
+      <c r="I35" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J35" s="80" t="inlineStr">
+        <is>
+          <t>No migrated data-layer decision exists yet; SDD must capture the chosen canonical account schema and any conversion rule.</t>
+        </is>
+      </c>
+      <c r="K35" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L35" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M35" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N35" s="80" t="inlineStr">
+        <is>
+          <t>No COBOL .specify/memory/constitution.md or specs/ SDD artifacts existed when this row was captured; constitution was added on 2026-07-09 and feature specs are still pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" collapsed="1" ht="66" customHeight="1">
+      <c r="A36" s="77" t="inlineStr">
+        <is>
+          <t>UF-006</t>
+        </is>
+      </c>
+      <c r="B36" s="77" t="inlineStr">
+        <is>
+          <t>Legacy Runtime &amp; Demo Deployment</t>
+        </is>
+      </c>
+      <c r="C36" s="77" t="inlineStr">
+        <is>
+          <t>Not Passed - Missed</t>
+        </is>
+      </c>
+      <c r="D36" s="77" t="inlineStr">
+        <is>
+          <t>Dockerized legacy runtime exists for evidence gathering, but no migration SDD or target runtime decision exists yet.</t>
+        </is>
+      </c>
+      <c r="E36" s="77" t="n"/>
+      <c r="F36" s="77" t="n"/>
+      <c r="G36" s="77" t="n"/>
+      <c r="H36" s="77" t="n"/>
+      <c r="I36" s="77" t="n"/>
+      <c r="J36" s="77" t="n"/>
+      <c r="K36" s="77" t="n"/>
+      <c r="L36" s="77" t="n"/>
+      <c r="M36" s="77" t="n"/>
+      <c r="N36" s="77" t="n"/>
+    </row>
+    <row r="37" hidden="1" outlineLevel="1" ht="37.5" customHeight="1">
+      <c r="A37" s="78" t="n"/>
+      <c r="B37" s="79" t="inlineStr">
+        <is>
+          <t>Compile COBOL modules</t>
+        </is>
+      </c>
+      <c r="C37" s="78" t="inlineStr">
+        <is>
+          <t>Operational path</t>
+        </is>
+      </c>
+      <c r="D37" s="80" t="inlineStr">
+        <is>
+          <t>The demo runtime shall compile INIT-DB, TRANS-PROC, REPORT-GEN as modules and BANK-MAIN as the executable menu program.</t>
+        </is>
+      </c>
+      <c r="E37" s="80" t="inlineStr">
+        <is>
+          <t>A reviewer can rebuild the legacy baseline consistently without installing GnuCOBOL on Windows.</t>
+        </is>
+      </c>
+      <c r="F37" s="80" t="inlineStr">
+        <is>
+          <t>Docker build produces runnable COBOL artifacts inside the container.</t>
+        </is>
+      </c>
+      <c r="G37" s="80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" s="80" t="inlineStr">
+        <is>
+          <t>Dockerfile installs gnucobol/make and runs cobc -m INIT-DB.CBL, cobc -m TRANS-PROC.CBL, cobc -m REPORT-GEN.CBL, cobc -x BANK-MAIN.CBL.</t>
+        </is>
+      </c>
+      <c r="I37" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J37" s="80" t="inlineStr">
+        <is>
+          <t>No target deployment architecture exists for a migrated COBOL replacement yet.</t>
+        </is>
+      </c>
+      <c r="K37" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L37" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M37" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N37" s="80" t="inlineStr">
+        <is>
+          <t>No COBOL .specify/memory/constitution.md or specs/ SDD artifacts exist yet in this repo as of 2026-07-09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" hidden="1" outlineLevel="1" ht="66" customHeight="1">
+      <c r="A38" s="78" t="n"/>
+      <c r="B38" s="79" t="inlineStr">
+        <is>
           <t>Run interactive terminal demo</t>
         </is>
       </c>
-      <c r="C35" s="78" t="inlineStr">
+      <c r="C38" s="78" t="inlineStr">
         <is>
           <t>Operational path</t>
         </is>
       </c>
-      <c r="D35" s="80" t="inlineStr">
+      <c r="D38" s="80" t="inlineStr">
         <is>
           <t>The legacy baseline shall be runnable as an interactive terminal session through Docker Compose.</t>
         </is>
       </c>
-      <c r="E35" s="80" t="inlineStr">
+      <c r="E38" s="80" t="inlineStr">
         <is>
           <t>The team can manually verify golden behavior before writing SDD or modern code.</t>
         </is>
       </c>
-      <c r="F35" s="80" t="inlineStr">
+      <c r="F38" s="80" t="inlineStr">
         <is>
           <t>`docker compose run --rm core-banking` opens the same console menu used in local and server smoke tests.</t>
         </is>
       </c>
-      <c r="G35" s="80" t="inlineStr">
+      <c r="G38" s="80" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H35" s="80" t="inlineStr">
+      <c r="H38" s="80" t="inlineStr">
         <is>
           <t>docker-compose.yml service core-banking has stdin_open true, tty true, command ./BANK-MAIN; README.demo.md documents the manual flow.</t>
         </is>
       </c>
-      <c r="I35" s="80" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J35" s="80" t="inlineStr">
+      <c r="I38" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J38" s="80" t="inlineStr">
         <is>
           <t>No browser/API wrapper or migrated runtime exists yet.</t>
         </is>
       </c>
-      <c r="K35" s="80" t="inlineStr">
+      <c r="K38" s="80" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L35" s="80" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M35" s="80" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="N35" s="80" t="inlineStr">
+      <c r="L38" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M38" s="80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N38" s="80" t="inlineStr">
         <is>
           <t>No COBOL .specify/memory/constitution.md or specs/ SDD artifacts exist yet in this repo as of 2026-07-09.</t>
         </is>
       </c>
     </row>
-    <row r="36" hidden="1" outlineLevel="1" ht="66" customHeight="1"/>
-    <row r="37" collapsed="1" ht="37.5" customHeight="1"/>
-    <row r="38" hidden="1" outlineLevel="1" ht="66" customHeight="1"/>
     <row r="39" hidden="1" outlineLevel="1" ht="66" customHeight="1"/>
     <row r="40" hidden="1" outlineLevel="1" ht="66" customHeight="1"/>
     <row r="41" hidden="1" outlineLevel="1" ht="66" customHeight="1"/>
@@ -2710,7 +2912,7 @@
     <row r="110" hidden="1" outlineLevel="1" ht="66" customHeight="1"/>
     <row r="111" hidden="1" outlineLevel="1" ht="66" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A6:N35"/>
+  <autoFilter ref="A6:N38"/>
   <mergeCells count="5">
     <mergeCell ref="I5:K5"/>
     <mergeCell ref="A2:N2"/>

</xml_diff>